<commit_message>
removed warning from gpsBool
</commit_message>
<xml_diff>
--- a/Course_Materials/Soldering Kit Inventory and Costs.xlsx
+++ b/Course_Materials/Soldering Kit Inventory and Costs.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sophi\Desktop\scopazpriv\SeaLabCTDv2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sophi\Desktop\SeaLabMOS\Course_Materials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3AAAFDDC-A19F-4AB1-B432-A7669B00754D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C50BB8A2-2848-4275-BB11-8AF43DBCB487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="15634" xr2:uid="{8AE7241A-83DF-401A-B2D8-DC93CC12F151}"/>
   </bookViews>
@@ -39,10 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="48">
-  <si>
-    <t>Soldering Iron</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="57">
   <si>
     <t>https://www.adafruit.com/product/3685</t>
   </si>
@@ -183,6 +180,36 @@
   </si>
   <si>
     <t>Digital multimeter</t>
+  </si>
+  <si>
+    <t>Tip rinner</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/Thermaltronics-FBA_TMT-TC-2-Lead-Tinner-Container/dp/B00NS4J6BY</t>
+  </si>
+  <si>
+    <t>Desktop power supply</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/Adjustable-Switching-Regulated-Adjustments-Jesverty/dp/B09YSJQWRG</t>
+  </si>
+  <si>
+    <t>Soldering iron</t>
+  </si>
+  <si>
+    <t>Soldering iron stand</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/Soldering-Spring-Holder-Support-Station/dp/B08JLJLX4D</t>
+  </si>
+  <si>
+    <t>Tools</t>
+  </si>
+  <si>
+    <t>Consumables</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
   </si>
 </sst>
 </file>
@@ -193,7 +220,7 @@
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.0_);_(&quot;$&quot;* \(#,##0.0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -221,16 +248,29 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -238,25 +278,55 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -594,460 +664,565 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D98377C-B48C-44F1-8522-3296B92FD41F}">
-  <dimension ref="B1:J26"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.23046875" style="1"/>
     <col min="2" max="2" width="28.765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.69140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.69140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.23046875" style="1"/>
-    <col min="7" max="7" width="4.765625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="1.4609375" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="9.23046875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="B1" s="2" t="s">
+    <row r="1" spans="1:10" ht="15.45" x14ac:dyDescent="0.4">
+      <c r="A1" s="6"/>
+      <c r="B1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B2" s="1" t="s">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A2" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" s="11">
+        <v>20</v>
+      </c>
+      <c r="D2" s="12">
+        <v>1</v>
+      </c>
+      <c r="E2" s="11">
+        <f t="shared" ref="E2:E15" si="0">C2*D2</f>
+        <v>20</v>
+      </c>
+      <c r="F2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="5">
-        <v>20</v>
-      </c>
-      <c r="D2" s="6">
-        <v>1</v>
-      </c>
-      <c r="E2" s="5">
-        <f t="shared" ref="E2:E13" si="0">C2*D2</f>
-        <v>20</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="G2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="H2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A3" s="10"/>
+      <c r="B3" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3" s="11">
+        <v>8</v>
+      </c>
+      <c r="D3" s="12">
+        <v>1</v>
+      </c>
+      <c r="E3" s="11">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I3" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B3" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" s="5">
+      <c r="J3" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A4" s="10"/>
+      <c r="B4" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="11">
         <v>10</v>
       </c>
-      <c r="D3" s="6">
-        <v>1</v>
-      </c>
-      <c r="E3" s="5">
+      <c r="D4" s="12">
+        <v>1</v>
+      </c>
+      <c r="E4" s="11">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="5">
+      <c r="F4" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A5" s="10"/>
+      <c r="B5" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="11">
         <v>7.25</v>
       </c>
-      <c r="D4" s="6">
-        <v>1</v>
-      </c>
-      <c r="E4" s="5">
+      <c r="D5" s="12">
+        <v>1</v>
+      </c>
+      <c r="E5" s="11">
         <f t="shared" si="0"/>
         <v>7.25</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B5" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="5">
+      <c r="F5" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A6" s="10"/>
+      <c r="B6" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="11">
         <v>17.5</v>
       </c>
-      <c r="D5" s="6">
-        <v>1</v>
-      </c>
-      <c r="E5" s="5">
+      <c r="D6" s="12">
+        <v>1</v>
+      </c>
+      <c r="E6" s="11">
         <f t="shared" si="0"/>
         <v>17.5</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B6" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" s="5">
+      <c r="F6" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A7" s="10"/>
+      <c r="B7" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="11">
         <v>12</v>
       </c>
-      <c r="D6" s="6">
-        <v>1</v>
-      </c>
-      <c r="E6" s="5">
+      <c r="D7" s="12">
+        <v>1</v>
+      </c>
+      <c r="E7" s="11">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B7" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C7" s="5">
+      <c r="F7" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" s="10"/>
+      <c r="B8" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="11">
         <v>3</v>
       </c>
-      <c r="D7" s="6">
-        <v>1</v>
-      </c>
-      <c r="E7" s="5">
+      <c r="D8" s="12">
+        <v>1</v>
+      </c>
+      <c r="E8" s="11">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F8" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" s="10"/>
+      <c r="B9" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="G7" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B8" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C8" s="5">
+      <c r="C9" s="11">
         <v>5</v>
       </c>
-      <c r="D8" s="6">
-        <v>1</v>
-      </c>
-      <c r="E8" s="5">
+      <c r="D9" s="12">
+        <v>1</v>
+      </c>
+      <c r="E9" s="11">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="F8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G8" s="1" t="s">
+      <c r="F9" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" s="10"/>
+      <c r="B10" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="11">
+        <v>5</v>
+      </c>
+      <c r="D10" s="12">
         <v>2</v>
       </c>
-    </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B9" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" s="5">
-        <v>5</v>
-      </c>
-      <c r="D9" s="6">
-        <v>2</v>
-      </c>
-      <c r="E9" s="5">
+      <c r="E10" s="11">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="F9" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B10" s="1" t="s">
+      <c r="F10" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" s="10"/>
+      <c r="B11" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="11">
         <v>27</v>
       </c>
-      <c r="C10" s="5">
-        <v>27</v>
-      </c>
-      <c r="D10" s="6">
-        <v>1</v>
-      </c>
-      <c r="E10" s="5">
+      <c r="D11" s="12">
+        <v>1</v>
+      </c>
+      <c r="E11" s="11">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="F10" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B11" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C11" s="5">
+      <c r="F11" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A12" s="10"/>
+      <c r="B12" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" s="11">
         <v>70</v>
       </c>
-      <c r="D11" s="6">
-        <v>1</v>
-      </c>
-      <c r="E11" s="5">
+      <c r="D12" s="12">
+        <v>1</v>
+      </c>
+      <c r="E12" s="11">
         <f t="shared" si="0"/>
         <v>70</v>
       </c>
-      <c r="F11" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B12" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C12" s="5">
+      <c r="F12" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13" s="10"/>
+      <c r="B13" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="11">
         <v>18</v>
       </c>
-      <c r="D12" s="6">
-        <v>1</v>
-      </c>
-      <c r="E12" s="5">
+      <c r="D13" s="12">
+        <v>1</v>
+      </c>
+      <c r="E13" s="11">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="F12" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B13" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C13" s="5">
+      <c r="F13" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A14" s="10"/>
+      <c r="B14" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="11">
         <v>15</v>
       </c>
-      <c r="D13" s="6">
-        <v>1</v>
-      </c>
-      <c r="E13" s="5">
+      <c r="D14" s="12">
+        <v>1</v>
+      </c>
+      <c r="E14" s="11">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="F13" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="G13" s="1" t="s">
+      <c r="F14" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A15" s="10"/>
+      <c r="B15" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" s="11">
+        <v>50</v>
+      </c>
+      <c r="D15" s="12">
+        <v>1</v>
+      </c>
+      <c r="E15" s="11">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="3" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="13"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="13"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A17" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17" s="11">
+        <v>27.5</v>
+      </c>
+      <c r="D17" s="12">
         <v>2</v>
       </c>
-    </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B15" s="1" t="s">
+      <c r="E17" s="11">
+        <f>C17*D17</f>
+        <v>55</v>
+      </c>
+      <c r="F17" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C15" s="5">
-        <v>27.5</v>
-      </c>
-      <c r="D15" s="6">
+      <c r="G17" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A18" s="10"/>
+      <c r="B18" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C18" s="11">
+        <v>6.5</v>
+      </c>
+      <c r="D18" s="12">
+        <v>1</v>
+      </c>
+      <c r="E18" s="11">
+        <f>C18*D18</f>
+        <v>6.5</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" s="10"/>
+      <c r="B19" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" s="11">
+        <v>3</v>
+      </c>
+      <c r="D19" s="12">
         <v>2</v>
       </c>
-      <c r="E15" s="5">
-        <f>C15*D15</f>
-        <v>55</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G15" s="1" t="s">
+      <c r="E19" s="11">
+        <f t="shared" ref="E19:E24" si="1">C19*D19</f>
+        <v>6</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A20" s="10"/>
+      <c r="B20" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" s="11">
+        <v>8</v>
+      </c>
+      <c r="D20" s="12">
         <v>2</v>
       </c>
-    </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B16" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C16" s="5">
-        <v>3</v>
-      </c>
-      <c r="D16" s="6">
-        <v>2</v>
-      </c>
-      <c r="E16" s="5">
-        <f t="shared" ref="E16:E21" si="1">C16*D16</f>
-        <v>6</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B17" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C17" s="5">
-        <v>8</v>
-      </c>
-      <c r="D17" s="6">
-        <v>2</v>
-      </c>
-      <c r="E17" s="5">
+      <c r="E20" s="11">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
-      <c r="F17" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B18" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C18" s="5">
+      <c r="F20" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" s="10"/>
+      <c r="B21" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="11">
         <v>5</v>
       </c>
-      <c r="D18" s="6">
+      <c r="D21" s="12">
         <v>3</v>
       </c>
-      <c r="E18" s="5">
+      <c r="E21" s="11">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G18" s="1" t="s">
+      <c r="F21" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" s="10"/>
+      <c r="B22" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="11">
+        <v>5</v>
+      </c>
+      <c r="D22" s="12">
         <v>2</v>
       </c>
-    </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B19" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C19" s="5">
-        <v>5</v>
-      </c>
-      <c r="D19" s="6">
-        <v>2</v>
-      </c>
-      <c r="E19" s="5">
+      <c r="E22" s="11">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="F19" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B20" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C20" s="5">
+      <c r="F22" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" s="10"/>
+      <c r="B23" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C23" s="11">
         <v>30</v>
       </c>
-      <c r="D20" s="6">
-        <v>1</v>
-      </c>
-      <c r="E20" s="5">
+      <c r="D23" s="12">
+        <v>1</v>
+      </c>
+      <c r="E23" s="11">
         <f t="shared" si="1"/>
         <v>30</v>
       </c>
-      <c r="F20" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B21" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C21" s="5">
-        <v>1</v>
-      </c>
-      <c r="D21" s="6">
+      <c r="F23" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" s="10"/>
+      <c r="B24" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" s="11">
+        <v>1</v>
+      </c>
+      <c r="D24" s="12">
         <v>4</v>
       </c>
-      <c r="E21" s="5">
+      <c r="E24" s="11">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="F21" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="E22" s="1"/>
-    </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="E26" s="5">
-        <f>SUM(E2:E21)</f>
-        <v>350.75</v>
+      <c r="F24" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="E25" s="1"/>
+    </row>
+    <row r="26" spans="1:7" ht="15.45" x14ac:dyDescent="0.4">
+      <c r="E26" s="4">
+        <f>SUM(E2:E24)</f>
+        <v>415.25</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:A15"/>
+    <mergeCell ref="A17:A24"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>